<commit_message>
fix(ifta): no reminder promise, fuller R245 wording, hedged quick check (review follow-up)
Independent review ACCEPT WITH FIXES:
- HIGH: the page promised IFTA deadline reminders the kit list doesn't send.
  It now says to put the due dates in your own calendar, that nothing here
  sends reminders, and that the kit list is for the kit announcement only.
  Test guards the wording.
- Workbook quick check: "Does not meet a QMV test" now says "on these
  numbers - confirm with your base jurisdiction before you skip IFTA";
  weight hints say use gross or registered, whichever is higher.
- "Who has to file": "used, designed or maintained" per R245; non-CDL FAQ
  adds whichever-is-higher weight and the two-jurisdiction trigger (R305).
- Rounding note: pennies to a few dollars, and rows vs total by a cent.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hotshot/downloads/hotshot-math-ifta-worksheet.xlsx
+++ b/hotshot/downloads/hotshot-math-ifta-worksheet.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jston\AppData\Local\Temp\claude\C--Users-jston-Vault\65110370-aabf-40b0-8298-a551f2aac95d\scratchpad\out\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\Repos\projectcalc-ifta-20261025\hotshot\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEBE76B8-5E4A-41CF-8BE7-8B44F550C41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E57594B0-DA79-4D3E-81D9-4D879ECBB758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3072" yWindow="3072" windowWidth="30960" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,21 +110,12 @@
     <t>Truck gross or registered weight (lb)</t>
   </si>
   <si>
-    <t>Gross vehicle weight or registered gross vehicle weight of the truck alone.</t>
-  </si>
-  <si>
     <t>Truck + trailer combination weight (lb)</t>
   </si>
   <si>
-    <t>Gross or registered weight of the whole combination. Leave blank if you run without a trailer.</t>
-  </si>
-  <si>
     <t>Result</t>
   </si>
   <si>
-    <t>Quick check only. 'Meets a QMV test' means IFTA reporting likely applies if you run in two or more member jurisdictions; ask your base jurisdiction to confirm.</t>
-  </si>
-  <si>
     <t>THINGS PEOPLE MISS</t>
   </si>
   <si>
@@ -354,6 +345,15 @@
   </si>
   <si>
     <t>Made by Hotshot Math. Provided as is, free to use and to share unchanged. Nothing here is affiliated with or endorsed by IFTA, Inc. or any government agency.</t>
+  </si>
+  <si>
+    <t>Gross vehicle weight or registered gross vehicle weight of the truck alone - use whichever is higher.</t>
+  </si>
+  <si>
+    <t>Gross or registered weight of the whole combination - use whichever is higher. Leave blank if you run without a trailer.</t>
+  </si>
+  <si>
+    <t>Quick check only. 'Meets a QMV test' means IFTA reporting likely applies if you run in two or more member jurisdictions. 'Does not meet' is not a ruling. Either way, ask your base jurisdiction to confirm.</t>
   </si>
 </sst>
 </file>
@@ -593,11 +593,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1069,38 +1069,38 @@
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="2" t="s">
-        <v>23</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B25" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C25" s="13"/>
       <c r="D25" s="2" t="s">
-        <v>25</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B26" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C26" s="50" t="str">
-        <f>IF(AND(N(C23)=0,N(C24)=0,N(C25)=0),"Enter your numbers",IF(OR(AND(N(C23)=2,N(C24)&gt;26000),N(C23)&gt;=3,N(C25)&gt;26000),"Meets a QMV test","Does not meet a QMV test"))</f>
+        <v>24</v>
+      </c>
+      <c r="C26" s="51" t="str">
+        <f>IF(AND(N(C23)=0,N(C24)=0,N(C25)=0),"Enter your numbers",IF(OR(AND(N(C23)=2,N(C24)&gt;26000),N(C23)&gt;=3,N(C25)&gt;26000),"Meets a QMV test","Does not meet a QMV test on these numbers - confirm with your base jurisdiction before you skip IFTA"))</f>
         <v>Enter your numbers</v>
       </c>
-      <c r="D26" s="51"/>
+      <c r="D26" s="52"/>
     </row>
     <row r="27" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="52" t="s">
-        <v>27</v>
+      <c r="B27" s="50" t="s">
+        <v>104</v>
       </c>
       <c r="C27" s="49"/>
       <c r="D27" s="49"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -1108,67 +1108,67 @@
     </row>
     <row r="30" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B30" s="48" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C30" s="49"/>
       <c r="D30" s="49"/>
     </row>
     <row r="31" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B31" s="48" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C31" s="49"/>
       <c r="D31" s="49"/>
     </row>
     <row r="32" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" s="48" t="s">
         <v>29</v>
-      </c>
-      <c r="B32" s="48" t="s">
-        <v>32</v>
       </c>
       <c r="C32" s="49"/>
       <c r="D32" s="49"/>
     </row>
     <row r="33" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B33" s="48" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C33" s="49"/>
       <c r="D33" s="49"/>
     </row>
     <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B34" s="48" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C34" s="49"/>
       <c r="D34" s="49"/>
     </row>
     <row r="35" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B35" s="48" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C35" s="49"/>
       <c r="D35" s="49"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -1176,59 +1176,52 @@
     </row>
     <row r="38" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="48" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C38" s="49"/>
       <c r="D38" s="15" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="48" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C39" s="49"/>
       <c r="D39" s="15" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="48" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C40" s="49"/>
       <c r="D40" s="15" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="48" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C41" s="49"/>
       <c r="D41" s="15" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B43" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B44" s="16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B27:D27"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B33:D33"/>
@@ -1240,11 +1233,18 @@
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B39:C39"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B39:C39"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" allowBlank="1" errorTitle="Axles" error="Enter a whole number of axles (1 to 12)." sqref="C23" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -1286,56 +1286,56 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="18" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B5" s="20">
         <v>2026</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B6" s="21">
         <f>IFERROR(INDEX('Due dates'!$E$6:$E$9,MATCH($B$4,'Due dates'!$A$6:$A$9,0)),"")</f>
         <v>46328</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B7" s="22">
         <f>IF(N($C$45)&gt;0,$B$45/$C$45,"")</f>
@@ -1344,16 +1344,16 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B8" s="23"/>
       <c r="C8" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="18" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B9" s="22">
         <f>IF(N($B$8)&gt;0,$B$8,IF(ISNUMBER($B$7),$B$7,""))</f>
@@ -1362,7 +1362,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="24" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B10" s="25" t="str">
         <f>IF(COUNT($F$15:$F$44)=0,"enter rates",$G$45)</f>
@@ -1371,52 +1371,52 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="18" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B11" s="26">
         <f>SUMPRODUCT((((($B$15:$B$44&lt;&gt;"")+($C$15:$C$44&lt;&gt;""))&gt;0)*($F$15:$F$44="")))</f>
         <v>3</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="27" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="28" t="s">
+      <c r="E14" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="F14" s="28" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="G14" s="28" t="s">
         <v>69</v>
-      </c>
-      <c r="E14" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="G14" s="28" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="29" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B15" s="13">
         <v>3100</v>
@@ -1440,7 +1440,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B16" s="13">
         <v>1800</v>
@@ -1464,7 +1464,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="29" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B17" s="13">
         <v>1000</v>
@@ -1974,7 +1974,7 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B45" s="35">
         <f>SUM(B15:B44)</f>
@@ -2000,22 +2000,22 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2072,12 +2072,12 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="48" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B2" s="49"/>
       <c r="C2" s="49"/>
@@ -2087,47 +2087,47 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B3" s="26">
         <f>'Quarter worksheet'!$B$5</f>
         <v>2026</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="40" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="D5" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="E5" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="28" t="s">
-        <v>88</v>
-      </c>
       <c r="F5" s="28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="41" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C6" s="43">
         <f>DATE($B$3+0,4,30)</f>
@@ -2148,10 +2148,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="41" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B7" s="42" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C7" s="43">
         <f>DATE($B$3+0,7,31)</f>
@@ -2172,10 +2172,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="41" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B8" s="42" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C8" s="43">
         <f>DATE($B$3+0,10,31)</f>
@@ -2196,10 +2196,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="41" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B9" s="42" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C9" s="43">
         <f>DATE($B$3+1,1,31)</f>
@@ -2220,35 +2220,35 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="40" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="D13" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="28" t="s">
+      <c r="E13" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="C13" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="D13" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="E13" s="28" t="s">
-        <v>88</v>
-      </c>
       <c r="F13" s="28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="41" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B14" s="42" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C14" s="43">
         <f>DATE(($B$3+1)+0,4,30)</f>
@@ -2269,10 +2269,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="41" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B15" s="42" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C15" s="43">
         <f>DATE(($B$3+1)+0,7,31)</f>
@@ -2293,10 +2293,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="41" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B16" s="42" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C16" s="43">
         <f>DATE(($B$3+1)+0,10,31)</f>
@@ -2317,10 +2317,10 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="41" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B17" s="42" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C17" s="43">
         <f>DATE(($B$3+1)+1,1,31)</f>
@@ -2341,7 +2341,7 @@
     </row>
     <row r="19" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="48" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B19" s="49"/>
       <c r="C19" s="49"/>
@@ -2351,22 +2351,22 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="47" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2396,42 +2396,42 @@
   <sheetData>
     <row r="1" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>